<commit_message>
upload and forcast button succesfully displaying the output
</commit_message>
<xml_diff>
--- a/forecast_output.xlsx
+++ b/forecast_output.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,17 +429,32 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Forecast</t>
+          <t>BestModel</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Best_Model</t>
+          <t>BestValue</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Accuracy_%</t>
+          <t>ExpSmoothing</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Linear</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>MovingAvg</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>ForecastRunTime</t>
         </is>
       </c>
     </row>
@@ -454,16 +469,27 @@
           <t>2027-01-01</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>4288</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Linear</t>
-        </is>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>MovingAvg</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>5062.5</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>4288.86452392713</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4288.848484848486</v>
+      </c>
+      <c r="G2" t="n">
+        <v>5062.5</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:03:19</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -477,16 +503,27 @@
           <t>2027-02-01</t>
         </is>
       </c>
-      <c r="C3" t="n">
-        <v>4186</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Linear</t>
-        </is>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>MovingAvg</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>5062.5</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>4186.703843200802</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4186.68414918415</v>
+      </c>
+      <c r="G3" t="n">
+        <v>5062.5</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:03:19</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -500,91 +537,135 @@
           <t>2027-03-01</t>
         </is>
       </c>
-      <c r="C4" t="n">
-        <v>4084</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Linear</t>
-        </is>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>MovingAvg</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>5062.5</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>4084.543162474475</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4084.519813519814</v>
+      </c>
+      <c r="G4" t="n">
+        <v>5062.5</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:03:19</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Product B</t>
+          <t>Product A</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>5180</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Moving Average</t>
-        </is>
+          <t>2027-04-01</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>MovingAvg</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>5062.5</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>3982.382481748148</v>
+      </c>
+      <c r="F5" t="n">
+        <v>3982.355477855479</v>
+      </c>
+      <c r="G5" t="n">
+        <v>5062.5</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:03:19</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Product B</t>
+          <t>Product A</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2027-02-01</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>4780</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Moving Average</t>
-        </is>
+          <t>2027-05-01</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>MovingAvg</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>5062.5</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>3880.221801021821</v>
+      </c>
+      <c r="F6" t="n">
+        <v>3880.191142191143</v>
+      </c>
+      <c r="G6" t="n">
+        <v>5062.5</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:03:19</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Product B</t>
+          <t>Product A</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2027-03-01</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>5117</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Moving Average</t>
-        </is>
+          <t>2027-06-01</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MovingAvg</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>5062.5</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>3778.061120295494</v>
+      </c>
+      <c r="F7" t="n">
+        <v>3778.026806526807</v>
+      </c>
+      <c r="G7" t="n">
+        <v>5062.5</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:03:19</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Product C</t>
+          <t>Product B</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -592,22 +673,33 @@
           <t>2027-01-01</t>
         </is>
       </c>
-      <c r="C8" t="n">
-        <v>4221</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Linear</t>
-        </is>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ExpSmoothing</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>5309.760584934961</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>5309.760584934961</v>
+      </c>
+      <c r="F8" t="n">
+        <v>5309.712121212122</v>
+      </c>
+      <c r="G8" t="n">
+        <v>5015</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:03:19</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Product C</t>
+          <t>Product B</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -615,39 +707,367 @@
           <t>2027-02-01</t>
         </is>
       </c>
-      <c r="C9" t="n">
-        <v>4125</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Linear</t>
-        </is>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ExpSmoothing</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>5337.277477610823</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>5337.277477610823</v>
+      </c>
+      <c r="F9" t="n">
+        <v>5337.219114219115</v>
+      </c>
+      <c r="G9" t="n">
+        <v>5015</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:03:19</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Product B</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2027-03-01</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ExpSmoothing</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>5364.794370286684</v>
+      </c>
+      <c r="E10" t="n">
+        <v>5364.794370286684</v>
+      </c>
+      <c r="F10" t="n">
+        <v>5364.726107226108</v>
+      </c>
+      <c r="G10" t="n">
+        <v>5015</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:03:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Product B</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2027-04-01</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ExpSmoothing</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>5392.311262962546</v>
+      </c>
+      <c r="E11" t="n">
+        <v>5392.311262962546</v>
+      </c>
+      <c r="F11" t="n">
+        <v>5392.233100233101</v>
+      </c>
+      <c r="G11" t="n">
+        <v>5015</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:03:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Product B</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2027-05-01</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ExpSmoothing</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>5419.828155638407</v>
+      </c>
+      <c r="E12" t="n">
+        <v>5419.828155638407</v>
+      </c>
+      <c r="F12" t="n">
+        <v>5419.740093240093</v>
+      </c>
+      <c r="G12" t="n">
+        <v>5015</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:03:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Product B</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2027-06-01</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ExpSmoothing</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>5447.345048314269</v>
+      </c>
+      <c r="E13" t="n">
+        <v>5447.345048314269</v>
+      </c>
+      <c r="F13" t="n">
+        <v>5447.247086247086</v>
+      </c>
+      <c r="G13" t="n">
+        <v>5015</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:03:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>Product C</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2027-01-01</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>MovingAvg</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>4612.166666666667</v>
+      </c>
+      <c r="E14" t="n">
+        <v>4221.113092521507</v>
+      </c>
+      <c r="F14" t="n">
+        <v>4221.10606060606</v>
+      </c>
+      <c r="G14" t="n">
+        <v>4612.166666666667</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:03:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Product C</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2027-02-01</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>MovingAvg</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>4612.166666666667</v>
+      </c>
+      <c r="E15" t="n">
+        <v>4125.272065187217</v>
+      </c>
+      <c r="F15" t="n">
+        <v>4125.263403263403</v>
+      </c>
+      <c r="G15" t="n">
+        <v>4612.166666666667</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:03:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Product C</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
         <is>
           <t>2027-03-01</t>
         </is>
       </c>
-      <c r="C10" t="n">
-        <v>4029</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Linear</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>0</v>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>MovingAvg</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>4612.166666666667</v>
+      </c>
+      <c r="E16" t="n">
+        <v>4029.431037852926</v>
+      </c>
+      <c r="F16" t="n">
+        <v>4029.420745920746</v>
+      </c>
+      <c r="G16" t="n">
+        <v>4612.166666666667</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:03:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Product C</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2027-04-01</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>MovingAvg</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>4612.166666666667</v>
+      </c>
+      <c r="E17" t="n">
+        <v>3933.590010518636</v>
+      </c>
+      <c r="F17" t="n">
+        <v>3933.578088578089</v>
+      </c>
+      <c r="G17" t="n">
+        <v>4612.166666666667</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:03:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Product C</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2027-05-01</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>MovingAvg</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>4612.166666666667</v>
+      </c>
+      <c r="E18" t="n">
+        <v>3837.748983184345</v>
+      </c>
+      <c r="F18" t="n">
+        <v>3837.735431235431</v>
+      </c>
+      <c r="G18" t="n">
+        <v>4612.166666666667</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:03:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Product C</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2027-06-01</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>MovingAvg</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>4612.166666666667</v>
+      </c>
+      <c r="E19" t="n">
+        <v>3741.907955850054</v>
+      </c>
+      <c r="F19" t="n">
+        <v>3741.892773892774</v>
+      </c>
+      <c r="G19" t="n">
+        <v>4612.166666666667</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:03:19</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>